<commit_message>
feat: Added changing the names of files, queue handeling, config file changes.
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26731"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RPA\Claes\RoboticEnterpriseFramework-Windows\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RPA\Claes 2\RPA-Posthantering\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88E04312-470C-43F0-B9B2-655711C78DC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12570" activeTab="1"/>
+    <workbookView xWindow="5580" yWindow="1485" windowWidth="21600" windowHeight="11955" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="64">
   <si>
     <t>Name</t>
   </si>
@@ -84,9 +85,6 @@
   </si>
   <si>
     <t>logF_BusinessProcessName</t>
-  </si>
-  <si>
-    <t>Framework</t>
   </si>
   <si>
     <t>Orchestrator queue Name. The value must match with the queue name defined on Orchestrator.</t>
@@ -158,9 +156,6 @@
     <t xml:space="preserve">The maximum number of consecutive system exceptions was reached. </t>
   </si>
   <si>
-    <t>ProcessABCQueue</t>
-  </si>
-  <si>
     <t>Environment</t>
   </si>
   <si>
@@ -171,12 +166,63 @@
   </si>
   <si>
     <t>The number of retries to try to init all applications. To disable this feature, set the value to 0</t>
+  </si>
+  <si>
+    <t>Posthantering</t>
+  </si>
+  <si>
+    <t>Skannade filer</t>
+  </si>
+  <si>
+    <t>ApiGatewayDomainURL</t>
+  </si>
+  <si>
+    <t>EneoAppId</t>
+  </si>
+  <si>
+    <t>EneoVersion</t>
+  </si>
+  <si>
+    <t>Eneo_PollIntervalSeconds</t>
+  </si>
+  <si>
+    <t>Eneo_PollTimeoutSeconds</t>
+  </si>
+  <si>
+    <t>Eneo_MinConfidencePercent</t>
+  </si>
+  <si>
+    <t>EneoMinConfidencePercent</t>
+  </si>
+  <si>
+    <t>EneoPollIntervalSeconds</t>
+  </si>
+  <si>
+    <t>EneoPollTimeoutSeconds</t>
+  </si>
+  <si>
+    <t>Eneo_InputFolder</t>
+  </si>
+  <si>
+    <t>EneoInputFolder</t>
+  </si>
+  <si>
+    <t>Eneo_FileFilter</t>
+  </si>
+  <si>
+    <t>EneoFileFilter</t>
+  </si>
+  <si>
+    <t>Eneo_AppId</t>
+  </si>
+  <si>
+    <t>Eneo_Version</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4">
     <font>
       <sz val="11"/>
@@ -545,7 +591,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z998"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
@@ -591,22 +637,22 @@
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:26" ht="45">
       <c r="A3" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
@@ -615,15 +661,29 @@
         <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>47</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="7" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="7" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8">
+        <v>30</v>
+      </c>
+    </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
@@ -1622,7 +1682,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z989"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
@@ -1674,29 +1734,29 @@
         <v>0</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:26" ht="45">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="36" customHeight="1">
       <c r="A4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B4">
         <v>0</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:26" ht="14.25" customHeight="1"/>
@@ -1720,7 +1780,7 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
@@ -1742,7 +1802,7 @@
         <v>15</v>
       </c>
       <c r="C10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
@@ -1753,7 +1813,7 @@
         <v>17</v>
       </c>
       <c r="C11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
@@ -1764,53 +1824,53 @@
         <v>19</v>
       </c>
       <c r="C12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
       <c r="A13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B13" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B15">
         <v>2</v>
       </c>
       <c r="C15" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
       <c r="A16" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B16">
         <v>2</v>
       </c>
       <c r="C16" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="18" spans="1:3" ht="45">
       <c r="A18" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B18" t="b">
         <v>0</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="14.25" customHeight="1"/>
@@ -2792,7 +2852,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:Z1000"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
@@ -2810,7 +2870,7 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>4</v>
@@ -2840,23 +2900,79 @@
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
       <c r="A2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="5" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="7" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="3" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A4" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A5" t="s">
+        <v>63</v>
+      </c>
+      <c r="B5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A6" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A9" t="s">
+        <v>58</v>
+      </c>
+      <c r="B9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A10" t="s">
+        <v>60</v>
+      </c>
+      <c r="B10" t="s">
+        <v>61</v>
+      </c>
+    </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
@@ -3850,5 +3966,6 @@
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: can run i backgrund, new longer timeout time.
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RPA\Claes 2\RPA-Posthantering\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B9CA6D6-D277-4812-810D-79C9B1264681}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D25450E-EAB1-49DE-B57A-C56CE3476236}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5580" yWindow="1485" windowWidth="21600" windowHeight="11955" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -699,7 +699,7 @@
         <v>12</v>
       </c>
       <c r="B8">
-        <v>120</v>
+        <v>300</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>